<commit_message>
fix(figures): eliminate duplicate figures, standardize 12 unique technical images, sync to reports/figures and align supervisor report
</commit_message>
<xml_diff>
--- a/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Báo Cáo Tiến Độ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Checklist Tiến Độ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Nhật Ký Họp" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -137,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -177,6 +178,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -776,10 +780,10 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Khởi động &amp; Sàng lọc Papers:
-- Họp GVHD Meeting 1 (29/08) &amp; Meeting 2 (01/09).
-- Đọc &amp; sàng lọc 10 papers theo Register.
-- Cập nhật cơ sở lý thuyết Chapter 1&amp;2.</t>
+          <t>Khởi động, Papers &amp; Thiết kế Slide:
+- Tham gia Meeting 1 (29/08), Meeting 2 (01/09) &amp; Meeting 3 (08/09).
+- Cùng Đức trực tiếp thiết kế đồ họa, biên soạn nội dung và hoàn thiện bộ Slide 22 trang (PI-GUARD-Present-109.pptx) báo cáo tiến độ gặp GVHD ngày 10/09.
+- Đọc &amp; sàng lọc 10 papers, cập nhật cơ sở lý thuyết Chapter 1&amp;2.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -928,10 +932,10 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Khảo sát ML &amp; JailGuard:
-- Tham gia Meeting 1 &amp; Meeting 2 (01/09).
-- Đọc &amp; phân tích JailGuard (TOSEM 2025).
-- Tìm hiểu Targeted Mutators Workflow.</t>
+          <t>Khảo sát ML &amp; Thiết kế Slide:
+- Tham gia Meeting 1 (29/08), Meeting 2 (01/09) &amp; Meeting 3 (08/09).
+- Cùng Trường trực tiếp thiết kế đồ họa, biên soạn nội dung và hoàn thiện bộ Slide 22 trang (PI-GUARD-Present-109.pptx) báo cáo tiến độ gặp GVHD ngày 10/09.
+- Phân tích TOSEM 2025 và nghiên cứu cơ chế TF-IDF Character N-Grams.</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1080,10 +1084,10 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Khảo sát RAP-ID &amp; BIPIA:
-- Tham gia Meeting 1 &amp; Meeting 2 (01/09).
-- Phân tích Pre-fill pass (RAP-ID) &amp; BIPIA.
-- Tìm cơ sở khoa học DeBERTa &lt; 600M.</t>
+          <t>Khảo sát Mô hình &amp; Phản biện Slide:
+- Tham gia Meeting 1 (29/08), Meeting 2 (01/09) &amp; Meeting 3 (08/09).
+- Thảo luận, phản biện đóng góp ý kiến kỹ thuật cho bộ slide do Trường &amp; Đức biên soạn.
+- Khảo sát RAP-ID, BIPIA và cơ chế Disentangled Attention DeBERTa-v3.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1232,10 +1236,10 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Khảo sát Jailbreak &amp; Do-Not-Answer:
-- Tham gia Meeting 1 &amp; Meeting 2 (01/09).
-- Phân loại 3 chiến thuật Jailbreak (Survey).
-- Khảo sát Do-Not-Answer &amp; Black-box def.</t>
+          <t>Khảo sát Y văn &amp; Phản biện Slide:
+- Tham gia Meeting 1 (29/08), Meeting 2 (01/09) &amp; Meeting 3 (08/09).
+- Thảo luận, phản biện đóng góp ý kiến kỹ thuật cho bộ slide do Trường &amp; Đức biên soạn.
+- Khảo sát Do-Not-Answer và xây dựng cấu trúc 3 câu hỏi nghiên cứu IEEE (RQ1-RQ3).</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1371,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1447,7 +1451,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Họp GVHD định hướng bài toán (Meeting 1_29_08) &amp; Sàng lọc 10 papers khoa học (Meeting 2_01_09)</t>
+          <t>Họp định hướng &amp; Sàng lọc Y văn (Meeting 1: 29/08, Meeting 2: 01/09, Meeting 3: 08/09)</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
@@ -1462,12 +1466,12 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Biên bản Meeting 1 &amp; Meeting 2.md</t>
+          <t>Biên bản Meeting 1, 2, 3.md</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>13/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1488,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Thu thập &amp; thẩm định 17 papers chuẩn IEEE &gt;= 2022 theo CAPSTONE REGISTER</t>
+          <t>Thiết kế, biên soạn nội dung và hoàn thiện bộ Slide 22 trang báo cáo tiến độ gặp GVHD ngày 10/09 (PI-GUARD-Present-109.pptx)</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1494,17 +1498,17 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Trường (Leader)</t>
+          <t>Trường &amp; Đức</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>References/ &amp; REFERENCES_LOG.md</t>
+          <t>reports/PI-GUARD-Present-109.pptx</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>13/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
     </row>
@@ -1516,32 +1520,32 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2 (14/09 - 20/09)</t>
+          <t>Tuần 1 (07/09 - 13/09)</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Soạn thảo Chapter 1: Background &amp; Problem Statement (Lỗ hổng Von Neumann NLP)</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Thu thập &amp; thẩm định 17 papers chuẩn IEEE &gt;= 2022 theo CAPSTONE REGISTER</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Trường</t>
+          <t>Trường (Leader)</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/</t>
+          <t>References/ &amp; REFERENCES_LOG.md</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>13/09/2026</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1562,7 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Phân loại Threat Taxonomy (Direct/Indirect Injection vs Jailbreak theo OWASP)</t>
+          <t>Soạn thảo Chapter 1: Background &amp; Problem Statement (Lỗ hổng Von Neumann NLP)</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -1568,7 +1572,7 @@
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Trường &amp; Đức</t>
+          <t>Trường</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -1578,7 +1582,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1599,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Threat Model (NIST AI 100-2e2025) &amp; Attack Surface (/v1/chat)</t>
+          <t>Phân loại Threat Taxonomy (Direct/Indirect Injection vs Jailbreak theo OWASP)</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -1605,17 +1609,17 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Đức</t>
+          <t>Trường &amp; Đức</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>workspaces/ducnq/</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1636,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế Kiến trúc bảo vệ 3 lớp &amp; Cơ chế phòng thủ độ bền Robustness</t>
+          <t>Xây dựng Threat Model (NIST AI 100-2e2025) &amp; Attack Surface (/v1/chat)</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -1652,7 +1656,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1673,7 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Soạn thảo 3 Câu hỏi nghiên cứu IEEE (RQ1-RQ3), 3 Gaps &amp; 4 Đóng góp mới</t>
+          <t>Thiết kế Kiến trúc bảo vệ 3 lớp &amp; Cơ chế phòng thủ độ bền Robustness</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -1679,17 +1683,17 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Phương</t>
+          <t>Đức</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>workspaces/phuongddd/</t>
+          <t>workspaces/ducnq/</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
     </row>
@@ -1701,12 +1705,12 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Tuần 3 (21/09 - 27/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Khảo sát SOTA Guardrails, Luận giải chọn mô hình &amp; Khảo sát 5 Target LLMs</t>
+          <t>Soạn thảo 3 Câu hỏi nghiên cứu IEEE (RQ1-RQ3), 3 Gaps &amp; 4 Đóng góp mới</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -1716,17 +1720,17 @@
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>Việt</t>
+          <t>Phương</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>workspaces/vietpmh/</t>
+          <t>workspaces/phuongddd/</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1747,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế Ma trận 4 Kịch bản Minh họa Đề bài (2x2: Vulnerable vs Proposed Protected)</t>
+          <t>Khảo sát SOTA Guardrails, Luận giải chọn mô hình &amp; Khảo sát 5 Target LLMs</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -1753,7 +1757,7 @@
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Việt &amp; Phương</t>
+          <t>Việt</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
@@ -1763,7 +1767,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1784,7 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Hoàn thiện toàn văn Report No.1: Introduction (Chapter 1 — 10% Process Mark)</t>
+          <t>Thiết kế Ma trận 4 Kịch bản Minh họa Đề bài (2x2: Vulnerable vs Proposed Protected)</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -1790,17 +1794,17 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Trường (Leader)</t>
+          <t>Việt &amp; Phương</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/</t>
+          <t>workspaces/vietpmh/</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1821,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Hoàn thiện toàn văn Report No.2: Literature Review (Chapter 2 — 25% Process Mark)</t>
+          <t>Hoàn thiện toàn văn Report No.1: Introduction (Chapter 1 — 10% Process Mark)</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -1827,7 +1831,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Trường &amp; Phương</t>
+          <t>Trường (Leader)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -1837,7 +1841,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1858,7 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế dàn ý slide 9 trang Review 1 Presentation Slides (Bao gồm 2 Chương)</t>
+          <t>Hoàn thiện toàn văn Report No.2: Literature Review (Chapter 2 — 25% Process Mark)</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1864,7 +1868,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Phương</t>
+          <t>Trường &amp; Phương</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -1886,32 +1890,32 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Tuần 4 (28/09 - 04/10)</t>
+          <t>Tuần 3 (21/09 - 27/09)</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế slide PowerPoint (.pptx) &amp; Tập dượt thuyết trình 15 phút (2 Chương)</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+          <t>Thiết kế dàn ý slide 9 trang Review 1 Presentation Slides (Bao gồm 2 Chương)</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Cả 4 thành viên</t>
+          <t>Phương</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Slide PPTX Review 1</t>
+          <t>workspaces/truongnv/docs/</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>27/09/2026</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1932,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Họp tổng kết tuần, cập nhật Process Report Excel &amp; Nộp Report 1 &amp; 2 cho GVHD</t>
+          <t>Thiết kế slide PowerPoint (.pptx) &amp; Tập dượt thuyết trình 15 phút (2 Chương)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -1938,17 +1942,17 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Trường (Leader)</t>
+          <t>Cả 4 thành viên</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>PI_GUARD_PROCESS_REPORT.xlsx</t>
+          <t>Slide PPTX Review 1</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1969,7 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 1 — BẢO VỆ REVIEW 1 TRƯỚC GVHD (CHAPTERS 1 &amp; 2)</t>
+          <t>Họp tổng kết tuần, cập nhật Process Report Excel &amp; Nộp Report 1 &amp; 2 cho GVHD</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -1975,17 +1979,17 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Cả 4 thành viên</t>
+          <t>Trường (Leader)</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Biên bản nghiệm thu Review 1</t>
+          <t>PI_GUARD_PROCESS_REPORT.xlsx</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
     </row>
@@ -1997,12 +2001,12 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
+          <t>Tuần 4 (28/09 - 04/10)</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Thu thập Dataset đa nguồn, Group-Aware Split &amp; Huấn luyện Baseline ML</t>
+          <t>CỘT MỐC 1 — BẢO VỆ REVIEW 1 TRƯỚC GVHD (CHAPTERS 1 &amp; 2)</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -2012,17 +2016,17 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Trường &amp; Đức</t>
+          <t>Cả 4 thành viên</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>data/processed/ &amp; models/baseline/</t>
+          <t>Biên bản nghiệm thu Review 1</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>18/10/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2038,12 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Tuần 7 (19/10 - 25/10)</t>
+          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Soạn thảo, cập nhật docs Chapter 3 (Methodology - Report No.3) &amp; Chuẩn bị Slide Review 2</t>
+          <t>Thu thập Dataset đa nguồn, Group-Aware Split &amp; Huấn luyện Baseline ML</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -2049,17 +2053,17 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Đức &amp; Trường</t>
+          <t>Trường &amp; Đức</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>docs/thesis/chapters/03_Methodology.md &amp; Slide Review 2</t>
+          <t>data/processed/ &amp; models/baseline/</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>18/10/2026</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2075,12 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Tuần 8 (26/10 - 01/11)</t>
+          <t>Tuần 7 (19/10 - 25/10)</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 2 — BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3), Nộp Report No.3 &amp; Cập nhật Docs hoàn chỉnh</t>
+          <t>Soạn thảo, cập nhật docs Chapter 3 (Methodology - Report No.3) &amp; Chuẩn bị Slide Review 2</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
@@ -2086,17 +2090,17 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Cả 4 thành viên</t>
+          <t>Đức &amp; Trường</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Biên bản nghiệm thu Review 2 &amp; Chapter 3 final</t>
+          <t>docs/thesis/chapters/03_Methodology.md &amp; Slide Review 2</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>01/11/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2108,12 +2112,12 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Tuần 9 - 10 (02/11 - 15/11)</t>
+          <t>Tuần 8 (26/10 - 01/11)</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Fine-tuning DeBERTa-v3, Lượng hóa ONNX INT8, Đánh giá Adversarial &amp; Nộp Report No.4</t>
+          <t>CỘT MỐC 2 — BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3), Nộp Report No.3 &amp; Cập nhật Docs hoàn chỉnh</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -2123,17 +2127,17 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Việt &amp; Đức</t>
+          <t>Cả 4 thành viên</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Report No.4 &amp; models/onnx/</t>
+          <t>Biên bản nghiệm thu Review 2 &amp; Chapter 3 final</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>15/11/2026</t>
+          <t>01/11/2026</t>
         </is>
       </c>
     </row>
@@ -2145,12 +2149,12 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Tuần 11 - 12 (16/11 - 29/11)</t>
+          <t>Tuần 9 - 10 (02/11 - 15/11)</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng API Middleware, Streamlit Dashboard &amp; Tích hợp Prototype Demo 3 lớp</t>
+          <t>Fine-tuning DeBERTa-v3, Lượng hóa ONNX INT8, Đánh giá Adversarial &amp; Nộp Report No.4</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -2160,17 +2164,17 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Phương &amp; Việt</t>
+          <t>Việt &amp; Đức</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Hệ thống Prototype hoàn chỉnh</t>
+          <t>Report No.4 &amp; models/onnx/</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>29/11/2026</t>
+          <t>15/11/2026</t>
         </is>
       </c>
     </row>
@@ -2182,12 +2186,12 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Tuần 13 (30/11 - 06/12)</t>
+          <t>Tuần 11 - 12 (16/11 - 29/11)</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 3 — BÁO CÁO HỘI ĐỒNG 1 (HỘI ĐỒNG GIỮA KỲ — PROTOTYPE DEMO &amp; CHAPTER 4)</t>
+          <t>Xây dựng API Middleware, Streamlit Dashboard &amp; Tích hợp Prototype Demo 3 lớp</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
@@ -2197,17 +2201,17 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Cả 4 thành viên</t>
+          <t>Phương &amp; Việt</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Biên bản nghiệm thu Hội đồng 1</t>
+          <t>Hệ thống Prototype hoàn chỉnh</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>06/12/2026</t>
+          <t>29/11/2026</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2223,12 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Tuần 14 (07/12 - 13/12)</t>
+          <t>Tuần 13 (30/11 - 06/12)</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Soạn Report No.5 &amp; No.6, Tổng hợp Master Thesis 6 chương qua script &amp; Quét Turnitin (&lt; 20%)</t>
+          <t>CỘT MỐC 3 — BÁO CÁO HỘI ĐỒNG 1 (HỘI ĐỒNG GIỮA KỲ — PROTOTYPE DEMO &amp; CHAPTER 4)</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
@@ -2239,12 +2243,12 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>FINAL_THESIS.md &amp; Report 5, 6</t>
+          <t>Biên bản nghiệm thu Hội đồng 1</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>13/12/2026</t>
+          <t>06/12/2026</t>
         </is>
       </c>
     </row>
@@ -2256,30 +2260,67 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
+          <t>Tuần 14 (07/12 - 13/12)</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Soạn Report No.5 &amp; No.6, Tổng hợp Master Thesis 6 chương qua script &amp; Quét Turnitin (&lt; 20%)</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Cả 4 thành viên</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>FINAL_THESIS.md &amp; Report 5, 6</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>13/12/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
           <t>Tuần 15 (14/12 - 20/12)</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>CỘT MỐC 4 — BẢO VỆ TỐT NGHIỆP TOÀN DIỆN 6 CHƯƠNG TRƯỚC HỘI ĐỒNG FINAL</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Cả 4 thành viên</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Final Thesis &amp; Slide Defense</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>20/12/2026</t>
         </is>
@@ -2297,4 +2338,200 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NHẬT KÝ CÁC CUỘC HỌP VỚI GVHD &amp; HỌP NHÓM NỘI BỘ (PI-GUARD MEETING LOG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Học kỳ Fall 2026 (07/09/2026 – 20/12/2026) | Khoa An toàn Thông tin - Đại học FPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Mã cuộc họp</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Thời gian</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Hình thức / Địa điểm</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Thành phần tham dự</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Chủ đề &amp; Nội dung cốt lõi</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Phân công nhiệm vụ cụ thể &amp; Sản phẩm đầu ra</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Trạng thái &amp; Biên bản lưu trữ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Meet 01</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Trực tuyến (Google Meet với GVHD)</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Họp GVHD định hướng bài toán an ninh LLM</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Cả nhóm cùng thu thập tài liệu theo CAPSTONE REGISTER; Trường điều phối hồ sơ.
+Đầu ra: Meeting 1_29_08_26.md</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Hoàn thành (100%)
+Meeting/Meeting 1_29_08_26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Meet 02</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Trực tuyến qua Discord</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Cả 4 thành viên (Trường, Đức, Việt, Phương)</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Đọc hiểu, đánh giá khắt khe và sàng lọc các bài báo khoa học đã thu thập; kiên quyết loại bỏ bài báo ngoài phạm vi (như RAP-ID can thiệp KV-cache nội tại LLM) và bài báo trùng lặp.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Cả nhóm cùng tìm hiểu cơ chế hoạt động của 2 hướng mô hình (Baseline TF-IDF và Transformer DeBERTa-v3) trong workspace cá nhân.
+Đầu ra: Meeting 2_01_09_26.md.</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Hoàn thành (100%)
+Meeting/Meeting 2_01_09_26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Meet 03</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Trực tuyến qua Discord</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Cả 4 thành viên (Trường, Đức, Việt, Phương)</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Đánh giá kết quả nghiên cứu tuần 2 của 4 thành viên; chốt cấu trúc 3 phần và nội dung tạo slide thuyết trình phục vụ buổi gặp báo cáo tiến độ với GVHD ngày 10/09/2026.</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Trường và Đức trực tiếp phụ trách tạo slide, biên soạn nội dung và hoàn thiện toàn bộ bộ Slide 22 trang (PI-GUARD-Present-109.pptx).
+Đầu ra: Meeting 3_08_09_26.md &amp; reports/PI-GUARD-Present-109.pptx.</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Hoàn thành (100%)
+Meeting/Meeting 3_08_09_26.md
+reports/PI-GUARD-Present-109.pptx</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(meeting): update meeting 3 attendee roles, prune redundant sections, move FAQ to end of supervisor report
</commit_message>
<xml_diff>
--- a/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -1084,9 +1084,9 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Khảo sát Mô hình &amp; Phản biện Slide:
+          <t>Khảo sát Mô hình &amp; Rà soát Slide:
 - Tham gia Meeting 1 (29/08), Meeting 2 (01/09) &amp; Meeting 3 (08/09).
-- Thảo luận, phản biện đóng góp ý kiến kỹ thuật cho bộ slide do Trường &amp; Đức biên soạn.
+- Rà soát toàn bộ bộ slide do Trường &amp; Đức chuẩn bị, thống nhất 100% và không có ý kiến bổ sung.
 - Khảo sát RAP-ID, BIPIA và cơ chế Disentangled Attention DeBERTa-v3.</t>
         </is>
       </c>
@@ -1236,9 +1236,9 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Khảo sát Y văn &amp; Phản biện Slide:
+          <t>Khảo sát Y văn &amp; Rà soát Slide:
 - Tham gia Meeting 1 (29/08), Meeting 2 (01/09) &amp; Meeting 3 (08/09).
-- Thảo luận, phản biện đóng góp ý kiến kỹ thuật cho bộ slide do Trường &amp; Đức biên soạn.
+- Rà soát toàn bộ bộ slide do Trường &amp; Đức chuẩn bị, thống nhất 100% và không có ý kiến bổ sung.
 - Khảo sát Do-Not-Answer và xây dựng cấu trúc 3 câu hỏi nghiên cứu IEEE (RQ1-RQ3).</t>
         </is>
       </c>
@@ -2510,12 +2510,12 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Đánh giá kết quả nghiên cứu tuần 2 của 4 thành viên; chốt cấu trúc 3 phần và nội dung tạo slide thuyết trình phục vụ buổi gặp báo cáo tiến độ với GVHD ngày 10/09/2026.</t>
+          <t>Đánh giá kết quả nghiên cứu và thống nhất slide báo cáo tiến độ gặp GVHD ngày 10/09/2026.</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Trường và Đức trực tiếp phụ trách tạo slide, biên soạn nội dung và hoàn thiện toàn bộ bộ Slide 22 trang (PI-GUARD-Present-109.pptx).
+          <t>Trường và Đức trực tiếp tạo slide, biên soạn nội dung và hoàn thiện toàn bộ bộ Slide 22 trang (PI-GUARD-Present-109.pptx); Việt và Phương rà soát, thống nhất hoàn toàn và không có ý kiến bổ sung.
 Đầu ra: Meeting 3_08_09_26.md &amp; reports/PI-GUARD-Present-109.pptx.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
refactor(repo): consolidate repository architecture into 3 primary divisions: reports, workspaces, and docs for github pages
</commit_message>
<xml_diff>
--- a/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -1540,7 +1540,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>References/ &amp; REFERENCES_LOG.md</t>
+          <t>reports/References/ &amp; REFERENCES_LOG.md</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -2444,7 +2444,7 @@
       <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
-Meeting/Meeting 1_29_08_26.md</t>
+reports/Meeting/Meeting 1_29_08_26.md</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
-Meeting/Meeting 2_01_09_26.md</t>
+reports/Meeting/Meeting 2_01_09_26.md</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
-Meeting/Meeting 3_08_09_26.md
+reports/Meeting/Meeting 3_08_09_26.md
 reports/PI-GUARD-Present-109.pptx</t>
         </is>
       </c>

</xml_diff>